<commit_message>
Rename "Discovery" curriculum to "Introductory"
</commit_message>
<xml_diff>
--- a/static/standards-correlations/Alabama_CS1_State_Standards.xlsx
+++ b/static/standards-correlations/Alabama_CS1_State_Standards.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crosswalk" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Attribution" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Crosswalk" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Legend &amp; Attribution" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Crosswalk'!$A$4:$I$49</definedName>
@@ -565,10 +565,11 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scored against full lab bodies | C and Python tracks | Discovery Projects | 2025 Alabama Course of Study</t>
-        </is>
-      </c>
-    </row>
+          <t>Scored against full lab bodies | C and Python tracks | Introductory Projects | 2025 Alabama Course of Study</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -602,7 +603,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Discovery Projects</t>
+          <t>Introductory Projects</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -1097,7 +1098,7 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Unit 5.1 is built entirely around the second attempt. Discovery Systems 5 teaches define-brainstorm-build-test-improve explicitly.</t>
+          <t>Unit 5.1 is built entirely around the second attempt. Introductory Systems 5 teaches define-brainstorm-build-test-improve explicitly.</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2123,7 @@
       </c>
       <c r="I38" s="8" t="inlineStr">
         <is>
-          <t>Discovery Coding 2 notes that professional programmers spend most of their time debugging; Ext 5.3H (Find the Community) exposes students to real practitioner repositories.</t>
+          <t>Introductory Coding 2 notes that professional programmers spend most of their time debugging; Ext 5.3H (Find the Community) exposes students to real practitioner repositories.</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2534,7 @@
       </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>Discovery Systems 11 covers living well online. Ext 5.3D (Who's Left Out?) touches access pressure. Mental health risk investigation is absent.</t>
+          <t>Introductory Systems 11 covers living well online. Ext 5.3D (Who's Left Out?) touches access pressure. Mental health risk investigation is absent.</t>
         </is>
       </c>
     </row>
@@ -2657,6 +2658,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -2701,7 +2703,7 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Discovery Project, Coding strand, project NN (01-17).</t>
+          <t>Introductory Project, Coding strand, project NN (01-17).</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2715,7 @@
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Discovery Project, Systems strand, project NN (01-14).</t>
+          <t>Introductory Project, Systems strand, project NN (01-14).</t>
         </is>
       </c>
     </row>
@@ -2813,6 +2815,8 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
@@ -2828,7 +2832,7 @@
 SUPERSEDES the 2018 Alabama DLCS Course of Study.
 Crosswalk analysis (c) KIPR / Botball Explorer.
 === METHODOLOGY (revised) ===
-This crosswalk scores against FULL LAB BODIES: reflection prompts, Individual Reflection phases, AI Literacy Bridge sections, and Extension Challenges. Evidence base is 750 reflection prompts and 255 Extension Challenges across 27 C labs, 27 Python labs, and 31 Discovery projects.
+This crosswalk scores against FULL LAB BODIES: reflection prompts, Individual Reflection phases, AI Literacy Bridge sections, and Extension Challenges. Evidence base is 750 reflection prompts and 255 Extension Challenges across 27 C labs, 27 Python labs, and 31 Introductory projects.
 An earlier revision of this file scored lab FRONT MATTER ONLY (headings, descriptions, concept tags, objectives) and materially undercounted coverage. Those figures are superseded.
 Scoring rule: Full requires evidence in the core lab flow. Partial is assigned where the only evidence sits in an optional Extension Challenge (labelled 'Finished early?' in the labs), or where the standard is only partly met. Cells citing 'Ext N.NL' identify the specific extension carrying the evidence, so a reviewer can verify placement and decide whether optional work counts for their purposes.</t>
         </is>

</xml_diff>